<commit_message>
dados: 2026-10-12 14:58 (108 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Jul_2026.xlsx
+++ b/xlsx/carteira_mensal/Jul_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="123">
   <si>
     <t>Acompanhamento de Carteira</t>
   </si>
@@ -75,24 +75,24 @@
     <t>Data de Criação do Projeto</t>
   </si>
   <si>
+    <t>/  /     até   /  /</t>
+  </si>
+  <si>
+    <t>Data de Criação do Orçamento</t>
+  </si>
+  <si>
+    <t>/  /     00:00 até   /  /     00:00</t>
+  </si>
+  <si>
+    <t>Data de Criação do Contrato</t>
+  </si>
+  <si>
+    <t>Data de Assinatura do Contrato</t>
+  </si>
+  <si>
     <t>01/07/2026 até 31/07/2026</t>
   </si>
   <si>
-    <t>Data de Criação do Orçamento</t>
-  </si>
-  <si>
-    <t>/  /     00:00 até   /  /     00:00</t>
-  </si>
-  <si>
-    <t>Data de Criação do Contrato</t>
-  </si>
-  <si>
-    <t>/  /     até   /  /</t>
-  </si>
-  <si>
-    <t>Data de Assinatura do Contrato</t>
-  </si>
-  <si>
     <t>Data de Criação do Cliente</t>
   </si>
   <si>
@@ -153,24 +153,33 @@
     <t>Contrato</t>
   </si>
   <si>
+    <t>Marina Pezzotti Marques</t>
+  </si>
+  <si>
+    <t>Parceiro</t>
+  </si>
+  <si>
+    <t>17/06/26</t>
+  </si>
+  <si>
+    <t>ROSANGELA PACHECO</t>
+  </si>
+  <si>
+    <t>Orçamento 1</t>
+  </si>
+  <si>
+    <t>27/07/26</t>
+  </si>
+  <si>
     <t>Rafael Martins Sardinha</t>
   </si>
   <si>
-    <t>Parceiro</t>
-  </si>
-  <si>
     <t>02/07/26</t>
   </si>
   <si>
-    <t>ROSANGELA PACHECO</t>
-  </si>
-  <si>
     <t>Orçamento Principal</t>
   </si>
   <si>
-    <t>27/07/26</t>
-  </si>
-  <si>
     <t>Daniel Teixeira</t>
   </si>
   <si>
@@ -180,9 +189,6 @@
     <t>ERIC SERPA</t>
   </si>
   <si>
-    <t>Orçamento 1</t>
-  </si>
-  <si>
     <t>06/07/26</t>
   </si>
   <si>
@@ -333,7 +339,7 @@
     <t>Quantidade de Projetos</t>
   </si>
   <si>
-    <t>21</t>
+    <t>22</t>
   </si>
   <si>
     <t>Quantidade de Orçamentos</t>
@@ -342,40 +348,40 @@
     <t>Pontuação Total</t>
   </si>
   <si>
-    <t>1.92</t>
+    <t>1.93</t>
   </si>
   <si>
     <t>Valor Total Bruto</t>
   </si>
   <si>
-    <t>941.558,81</t>
-  </si>
-  <si>
-    <t>657.783,44</t>
+    <t>1.069.425,70</t>
+  </si>
+  <si>
+    <t>752.783,44</t>
   </si>
   <si>
     <t>Valor Total Líquido</t>
   </si>
   <si>
-    <t>614.785,72</t>
+    <t>702.876,41</t>
   </si>
   <si>
     <t>Total Líquido sem o Per</t>
   </si>
   <si>
-    <t>611.786,80</t>
+    <t>689.117,12</t>
   </si>
   <si>
     <t>Total Diferença Financeira</t>
   </si>
   <si>
-    <t>42.997,72</t>
+    <t>49.907,03</t>
   </si>
   <si>
     <t>Total Adicional dos Ambientes</t>
   </si>
   <si>
-    <t>33.990,09</t>
+    <t>39.308,69</t>
   </si>
 </sst>
 </file>
@@ -444,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:O62"/>
+  <dimension ref="A2:O63"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="53.22265625" customWidth="true" bestFit="true"/>
@@ -572,15 +578,15 @@
         <v>23</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="20">
@@ -588,7 +594,7 @@
         <v>26</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -596,7 +602,7 @@
         <v>27</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -702,7 +708,7 @@
         <v>47</v>
       </c>
       <c r="C31" t="n">
-        <v>860.0</v>
+        <v>843.0</v>
       </c>
       <c r="D31" t="s">
         <v>48</v>
@@ -720,22 +726,22 @@
         <v>51</v>
       </c>
       <c r="I31" t="n">
-        <v>22665.4</v>
+        <v>95000.0</v>
       </c>
       <c r="J31" t="n">
-        <v>1068.34</v>
+        <v>6909.31</v>
       </c>
       <c r="K31" t="n">
-        <v>21597.06</v>
+        <v>88090.69</v>
       </c>
       <c r="L31" t="n">
-        <v>21597.06</v>
+        <v>77330.32</v>
       </c>
       <c r="M31" t="n">
-        <v>1.8</v>
+        <v>2.03</v>
       </c>
       <c r="N31" t="n">
-        <v>86002.0</v>
+        <v>84301.0</v>
       </c>
       <c r="O31" t="s">
         <v>51</v>
@@ -746,422 +752,422 @@
         <v>52</v>
       </c>
       <c r="B32" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" t="n">
+        <v>860.0</v>
+      </c>
+      <c r="D32" t="s">
         <v>53</v>
       </c>
-      <c r="C32" t="n">
-        <v>859.0</v>
-      </c>
-      <c r="D32" t="s">
-        <v>48</v>
-      </c>
       <c r="E32" t="s">
+        <v>49</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G32" t="s">
         <v>54</v>
       </c>
-      <c r="F32" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G32" t="s">
-        <v>55</v>
-      </c>
       <c r="H32" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="I32" t="n">
-        <v>38177.77</v>
+        <v>22665.4</v>
       </c>
       <c r="J32" t="n">
-        <v>987.17</v>
+        <v>1068.34</v>
       </c>
       <c r="K32" t="n">
-        <v>37190.6</v>
+        <v>21597.06</v>
       </c>
       <c r="L32" t="n">
-        <v>36349.34</v>
+        <v>21597.06</v>
       </c>
       <c r="M32" t="n">
-        <v>1.96</v>
+        <v>1.8</v>
       </c>
       <c r="N32" t="n">
-        <v>85901.0</v>
+        <v>86002.0</v>
       </c>
       <c r="O32" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" t="n">
+        <v>859.0</v>
+      </c>
+      <c r="D33" t="s">
+        <v>53</v>
+      </c>
+      <c r="E33" t="s">
+        <v>57</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G33" t="s">
+        <v>50</v>
+      </c>
+      <c r="H33" t="s">
         <v>58</v>
       </c>
-      <c r="B33" t="s">
-        <v>53</v>
-      </c>
-      <c r="C33" t="n">
-        <v>862.0</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="I33" t="n">
+        <v>38177.77</v>
+      </c>
+      <c r="J33" t="n">
+        <v>987.17</v>
+      </c>
+      <c r="K33" t="n">
+        <v>37190.6</v>
+      </c>
+      <c r="L33" t="n">
+        <v>36349.34</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="N33" t="n">
+        <v>85901.0</v>
+      </c>
+      <c r="O33" t="s">
         <v>59</v>
-      </c>
-      <c r="E33" t="s">
-        <v>49</v>
-      </c>
-      <c r="F33" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G33" t="s">
-        <v>55</v>
-      </c>
-      <c r="H33" t="s">
-        <v>60</v>
-      </c>
-      <c r="I33" t="n">
-        <v>11840.44</v>
-      </c>
-      <c r="J33" t="n">
-        <v>434.46</v>
-      </c>
-      <c r="K33" t="n">
-        <v>11405.98</v>
-      </c>
-      <c r="L33" t="n">
-        <v>11405.98</v>
-      </c>
-      <c r="M33" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="N33" t="n">
-        <v>86201.0</v>
-      </c>
-      <c r="O33" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
+        <v>60</v>
+      </c>
+      <c r="B34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" t="n">
+        <v>862.0</v>
+      </c>
+      <c r="D34" t="s">
+        <v>61</v>
+      </c>
+      <c r="E34" t="s">
+        <v>49</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G34" t="s">
+        <v>50</v>
+      </c>
+      <c r="H34" t="s">
         <v>62</v>
       </c>
-      <c r="B34" t="s">
+      <c r="I34" t="n">
+        <v>11840.44</v>
+      </c>
+      <c r="J34" t="n">
+        <v>434.46</v>
+      </c>
+      <c r="K34" t="n">
+        <v>11405.98</v>
+      </c>
+      <c r="L34" t="n">
+        <v>11405.98</v>
+      </c>
+      <c r="M34" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="N34" t="n">
+        <v>86201.0</v>
+      </c>
+      <c r="O34" t="s">
         <v>63</v>
-      </c>
-      <c r="C34" t="n">
-        <v>861.0</v>
-      </c>
-      <c r="D34" t="s">
-        <v>59</v>
-      </c>
-      <c r="E34" t="s">
-        <v>64</v>
-      </c>
-      <c r="F34" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="G34" t="s">
-        <v>65</v>
-      </c>
-      <c r="H34" t="s">
-        <v>66</v>
-      </c>
-      <c r="I34" t="n">
-        <v>1000.0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>48.92</v>
-      </c>
-      <c r="K34" t="n">
-        <v>951.08</v>
-      </c>
-      <c r="L34" t="n">
-        <v>951.08</v>
-      </c>
-      <c r="M34" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="N34" t="n">
-        <v>86102.0</v>
-      </c>
-      <c r="O34" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B35" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C35" t="n">
-        <v>872.0</v>
+        <v>861.0</v>
       </c>
       <c r="D35" t="s">
         <v>61</v>
       </c>
       <c r="E35" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F35" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="G35" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="H35" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I35" t="n">
-        <v>14700.0</v>
+        <v>1000.0</v>
       </c>
       <c r="J35" t="n">
-        <v>1420.24</v>
+        <v>48.92</v>
       </c>
       <c r="K35" t="n">
-        <v>13279.76</v>
+        <v>951.08</v>
       </c>
       <c r="L35" t="n">
-        <v>13279.76</v>
+        <v>951.08</v>
       </c>
       <c r="M35" t="n">
-        <v>1.96</v>
+        <v>3.3</v>
       </c>
       <c r="N35" t="n">
-        <v>87201.0</v>
+        <v>86102.0</v>
       </c>
       <c r="O35" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C36" t="n">
-        <v>873.0</v>
+        <v>872.0</v>
       </c>
       <c r="D36" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E36" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F36" t="n">
         <v>1.0</v>
       </c>
       <c r="G36" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="I36" t="n">
-        <v>26000.01</v>
+        <v>14700.0</v>
       </c>
       <c r="J36" t="n">
-        <v>667.09</v>
+        <v>1420.24</v>
       </c>
       <c r="K36" t="n">
-        <v>25332.92</v>
+        <v>13279.76</v>
       </c>
       <c r="L36" t="n">
-        <v>24731.18</v>
+        <v>13279.76</v>
       </c>
       <c r="M36" t="n">
-        <v>1.85</v>
+        <v>1.96</v>
       </c>
       <c r="N36" t="n">
-        <v>87301.0</v>
+        <v>87201.0</v>
       </c>
       <c r="O36" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
+        <v>70</v>
+      </c>
+      <c r="B37" t="s">
+        <v>71</v>
+      </c>
+      <c r="C37" t="n">
+        <v>873.0</v>
+      </c>
+      <c r="D37" t="s">
         <v>72</v>
       </c>
-      <c r="B37" t="s">
-        <v>63</v>
-      </c>
-      <c r="C37" t="n">
-        <v>876.0</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
+        <v>66</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G37" t="s">
+        <v>50</v>
+      </c>
+      <c r="H37" t="s">
         <v>73</v>
       </c>
-      <c r="E37" t="s">
-        <v>54</v>
-      </c>
-      <c r="F37" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G37" t="s">
-        <v>55</v>
-      </c>
-      <c r="H37" t="s">
-        <v>74</v>
-      </c>
       <c r="I37" t="n">
-        <v>34000.0</v>
+        <v>26000.01</v>
       </c>
       <c r="J37" t="n">
-        <v>1247.55</v>
+        <v>667.09</v>
       </c>
       <c r="K37" t="n">
-        <v>32752.45</v>
+        <v>25332.92</v>
       </c>
       <c r="L37" t="n">
-        <v>32752.45</v>
+        <v>24731.18</v>
       </c>
       <c r="M37" t="n">
-        <v>1.96</v>
+        <v>1.85</v>
       </c>
       <c r="N37" t="n">
-        <v>87601.0</v>
+        <v>87301.0</v>
       </c>
       <c r="O37" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" t="n">
+        <v>876.0</v>
+      </c>
+      <c r="D38" t="s">
         <v>75</v>
       </c>
-      <c r="B38" t="s">
-        <v>47</v>
-      </c>
-      <c r="C38" t="n">
-        <v>882.0</v>
-      </c>
-      <c r="D38" t="s">
-        <v>60</v>
-      </c>
       <c r="E38" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="F38" t="n">
         <v>1.0</v>
       </c>
       <c r="G38" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H38" t="s">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="I38" t="n">
-        <v>18388.0</v>
+        <v>34000.0</v>
       </c>
       <c r="J38" t="n">
-        <v>2735.99</v>
+        <v>1247.55</v>
       </c>
       <c r="K38" t="n">
-        <v>15652.01</v>
+        <v>32752.45</v>
       </c>
       <c r="L38" t="n">
-        <v>15652.01</v>
+        <v>32752.45</v>
       </c>
       <c r="M38" t="n">
-        <v>1.9</v>
+        <v>1.96</v>
       </c>
       <c r="N38" t="n">
-        <v>88201.0</v>
+        <v>87601.0</v>
       </c>
       <c r="O38" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="C39" t="n">
-        <v>881.0</v>
+        <v>882.0</v>
       </c>
       <c r="D39" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E39" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="F39" t="n">
         <v>1.0</v>
       </c>
       <c r="G39" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H39" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="I39" t="n">
-        <v>1480.0</v>
+        <v>18388.0</v>
       </c>
       <c r="J39" t="n">
-        <v>0.0</v>
+        <v>2735.99</v>
       </c>
       <c r="K39" t="n">
-        <v>1480.0</v>
+        <v>15652.01</v>
       </c>
       <c r="L39" t="n">
-        <v>1480.0</v>
+        <v>15652.01</v>
       </c>
       <c r="M39" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="N39" t="n">
-        <v>88101.0</v>
+        <v>88201.0</v>
       </c>
       <c r="O39" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
         <v>79</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="n">
+        <v>881.0</v>
+      </c>
+      <c r="D40" t="s">
+        <v>62</v>
+      </c>
+      <c r="E40" t="s">
         <v>80</v>
       </c>
-      <c r="C40" t="n">
-        <v>880.0</v>
-      </c>
-      <c r="D40" t="s">
-        <v>60</v>
-      </c>
-      <c r="E40" t="s">
-        <v>64</v>
-      </c>
       <c r="F40" t="n">
         <v>1.0</v>
       </c>
       <c r="G40" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H40" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="I40" t="n">
-        <v>16645.87</v>
+        <v>1480.0</v>
       </c>
       <c r="J40" t="n">
-        <v>4019.29</v>
+        <v>0.0</v>
       </c>
       <c r="K40" t="n">
-        <v>12626.58</v>
+        <v>1480.0</v>
       </c>
       <c r="L40" t="n">
-        <v>12626.58</v>
+        <v>1480.0</v>
       </c>
       <c r="M40" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
       <c r="N40" t="n">
-        <v>88001.0</v>
+        <v>88101.0</v>
       </c>
       <c r="O40" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
     </row>
     <row r="41">
@@ -1169,90 +1175,90 @@
         <v>81</v>
       </c>
       <c r="B41" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C41" t="n">
-        <v>886.0</v>
+        <v>880.0</v>
       </c>
       <c r="D41" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="E41" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="F41" t="n">
         <v>1.0</v>
       </c>
       <c r="G41" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H41" t="s">
-        <v>83</v>
+        <v>51</v>
       </c>
       <c r="I41" t="n">
-        <v>35716.8</v>
+        <v>16645.87</v>
       </c>
       <c r="J41" t="n">
-        <v>3546.5</v>
+        <v>4019.29</v>
       </c>
       <c r="K41" t="n">
-        <v>32170.3</v>
+        <v>12626.58</v>
       </c>
       <c r="L41" t="n">
-        <v>31420.53</v>
+        <v>12626.58</v>
       </c>
       <c r="M41" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="N41" t="n">
-        <v>88601.0</v>
+        <v>88001.0</v>
       </c>
       <c r="O41" t="s">
-        <v>83</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
+        <v>83</v>
+      </c>
+      <c r="B42" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" t="n">
+        <v>886.0</v>
+      </c>
+      <c r="D42" t="s">
         <v>84</v>
       </c>
-      <c r="B42" t="s">
-        <v>53</v>
-      </c>
-      <c r="C42" t="n">
-        <v>884.0</v>
-      </c>
-      <c r="D42" t="s">
-        <v>82</v>
-      </c>
       <c r="E42" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F42" t="n">
         <v>1.0</v>
       </c>
       <c r="G42" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H42" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="I42" t="n">
-        <v>102000.0</v>
+        <v>35716.8</v>
       </c>
       <c r="J42" t="n">
-        <v>12052.71</v>
+        <v>3546.5</v>
       </c>
       <c r="K42" t="n">
-        <v>89947.29</v>
+        <v>32170.3</v>
       </c>
       <c r="L42" t="n">
-        <v>89947.29</v>
+        <v>31420.53</v>
       </c>
       <c r="M42" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="N42" t="n">
-        <v>88401.0</v>
+        <v>88601.0</v>
       </c>
       <c r="O42" t="s">
         <v>85</v>
@@ -1263,140 +1269,140 @@
         <v>86</v>
       </c>
       <c r="B43" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C43" t="n">
-        <v>893.0</v>
+        <v>884.0</v>
       </c>
       <c r="D43" t="s">
+        <v>84</v>
+      </c>
+      <c r="E43" t="s">
+        <v>57</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G43" t="s">
+        <v>50</v>
+      </c>
+      <c r="H43" t="s">
+        <v>73</v>
+      </c>
+      <c r="I43" t="n">
+        <v>102000.0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>12052.71</v>
+      </c>
+      <c r="K43" t="n">
+        <v>89947.29</v>
+      </c>
+      <c r="L43" t="n">
+        <v>89947.29</v>
+      </c>
+      <c r="M43" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="N43" t="n">
+        <v>88401.0</v>
+      </c>
+      <c r="O43" t="s">
         <v>87</v>
-      </c>
-      <c r="E43" t="s">
-        <v>64</v>
-      </c>
-      <c r="F43" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G43" t="s">
-        <v>55</v>
-      </c>
-      <c r="H43" t="s">
-        <v>88</v>
-      </c>
-      <c r="I43" t="n">
-        <v>1930.0</v>
-      </c>
-      <c r="J43" t="n">
-        <v>55.77</v>
-      </c>
-      <c r="K43" t="n">
-        <v>1874.23</v>
-      </c>
-      <c r="L43" t="n">
-        <v>1874.23</v>
-      </c>
-      <c r="M43" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="N43" t="n">
-        <v>89301.0</v>
-      </c>
-      <c r="O43" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
+        <v>88</v>
+      </c>
+      <c r="B44" t="s">
+        <v>56</v>
+      </c>
+      <c r="C44" t="n">
+        <v>893.0</v>
+      </c>
+      <c r="D44" t="s">
         <v>89</v>
       </c>
-      <c r="B44" t="s">
+      <c r="E44" t="s">
+        <v>66</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G44" t="s">
+        <v>50</v>
+      </c>
+      <c r="H44" t="s">
         <v>90</v>
       </c>
-      <c r="C44" t="n">
-        <v>898.0</v>
-      </c>
-      <c r="D44" t="s">
-        <v>88</v>
-      </c>
-      <c r="E44" t="s">
-        <v>54</v>
-      </c>
-      <c r="F44" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G44" t="s">
-        <v>55</v>
-      </c>
-      <c r="H44" t="s">
-        <v>91</v>
-      </c>
       <c r="I44" t="n">
-        <v>35000.0</v>
+        <v>1930.0</v>
       </c>
       <c r="J44" t="n">
-        <v>1284.24</v>
+        <v>55.77</v>
       </c>
       <c r="K44" t="n">
-        <v>33715.76</v>
+        <v>1874.23</v>
       </c>
       <c r="L44" t="n">
-        <v>32909.61</v>
+        <v>1874.23</v>
       </c>
       <c r="M44" t="n">
-        <v>1.9</v>
+        <v>1.91</v>
       </c>
       <c r="N44" t="n">
-        <v>89801.0</v>
+        <v>89301.0</v>
       </c>
       <c r="O44" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
+        <v>91</v>
+      </c>
+      <c r="B45" t="s">
+        <v>92</v>
+      </c>
+      <c r="C45" t="n">
+        <v>898.0</v>
+      </c>
+      <c r="D45" t="s">
+        <v>90</v>
+      </c>
+      <c r="E45" t="s">
+        <v>57</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G45" t="s">
+        <v>50</v>
+      </c>
+      <c r="H45" t="s">
         <v>93</v>
       </c>
-      <c r="B45" t="s">
-        <v>63</v>
-      </c>
-      <c r="C45" t="n">
-        <v>901.0</v>
-      </c>
-      <c r="D45" t="s">
-        <v>94</v>
-      </c>
-      <c r="E45" t="s">
-        <v>64</v>
-      </c>
-      <c r="F45" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G45" t="s">
-        <v>55</v>
-      </c>
-      <c r="H45" t="s">
-        <v>51</v>
-      </c>
       <c r="I45" t="n">
-        <v>52950.0</v>
+        <v>35000.0</v>
       </c>
       <c r="J45" t="n">
-        <v>3328.95</v>
+        <v>1284.24</v>
       </c>
       <c r="K45" t="n">
-        <v>49621.05</v>
+        <v>33715.76</v>
       </c>
       <c r="L45" t="n">
-        <v>49621.05</v>
+        <v>32909.61</v>
       </c>
       <c r="M45" t="n">
         <v>1.9</v>
       </c>
       <c r="N45" t="n">
-        <v>90101.0</v>
+        <v>89801.0</v>
       </c>
       <c r="O45" t="s">
-        <v>51</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46">
@@ -1404,140 +1410,140 @@
         <v>95</v>
       </c>
       <c r="B46" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C46" t="n">
-        <v>900.0</v>
+        <v>901.0</v>
       </c>
       <c r="D46" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E46" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="F46" t="n">
         <v>1.0</v>
       </c>
       <c r="G46" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H46" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="I46" t="n">
-        <v>1100.0</v>
+        <v>52950.0</v>
       </c>
       <c r="J46" t="n">
-        <v>0.0</v>
+        <v>3328.95</v>
       </c>
       <c r="K46" t="n">
-        <v>1100.0</v>
+        <v>49621.05</v>
       </c>
       <c r="L46" t="n">
-        <v>1100.0</v>
+        <v>49621.05</v>
       </c>
       <c r="M46" t="n">
-        <v>3.0</v>
+        <v>1.9</v>
       </c>
       <c r="N46" t="n">
-        <v>90001.0</v>
+        <v>90101.0</v>
       </c>
       <c r="O46" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="B47" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C47" t="n">
-        <v>907.0</v>
+        <v>900.0</v>
       </c>
       <c r="D47" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="E47" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="F47" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="G47" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H47" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="I47" t="n">
-        <v>16223.15</v>
+        <v>1100.0</v>
       </c>
       <c r="J47" t="n">
-        <v>3917.2</v>
+        <v>0.0</v>
       </c>
       <c r="K47" t="n">
-        <v>12305.95</v>
+        <v>1100.0</v>
       </c>
       <c r="L47" t="n">
-        <v>12305.95</v>
+        <v>1100.0</v>
       </c>
       <c r="M47" t="n">
-        <v>1.8</v>
+        <v>3.0</v>
       </c>
       <c r="N47" t="n">
-        <v>90701.0</v>
+        <v>90001.0</v>
       </c>
       <c r="O47" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B48" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
       <c r="C48" t="n">
-        <v>905.0</v>
+        <v>907.0</v>
       </c>
       <c r="D48" t="s">
         <v>51</v>
       </c>
       <c r="E48" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F48" t="n">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="G48" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H48" t="s">
-        <v>98</v>
+        <v>51</v>
       </c>
       <c r="I48" t="n">
-        <v>18271.0</v>
+        <v>16223.15</v>
       </c>
       <c r="J48" t="n">
-        <v>1222.02</v>
+        <v>3917.2</v>
       </c>
       <c r="K48" t="n">
-        <v>17048.98</v>
+        <v>12305.95</v>
       </c>
       <c r="L48" t="n">
-        <v>17048.98</v>
+        <v>12305.95</v>
       </c>
       <c r="M48" t="n">
-        <v>1.91</v>
+        <v>1.8</v>
       </c>
       <c r="N48" t="n">
-        <v>90501.0</v>
+        <v>90701.0</v>
       </c>
       <c r="O48" t="s">
-        <v>98</v>
+        <v>51</v>
       </c>
     </row>
     <row r="49">
@@ -1545,93 +1551,93 @@
         <v>99</v>
       </c>
       <c r="B49" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="C49" t="n">
-        <v>904.0</v>
+        <v>905.0</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
       </c>
       <c r="E49" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F49" t="n">
         <v>1.0</v>
       </c>
       <c r="G49" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H49" t="s">
-        <v>51</v>
+        <v>100</v>
       </c>
       <c r="I49" t="n">
-        <v>181445.0</v>
+        <v>18271.0</v>
       </c>
       <c r="J49" t="n">
-        <v>3852.58</v>
+        <v>1222.02</v>
       </c>
       <c r="K49" t="n">
-        <v>177592.42</v>
+        <v>17048.98</v>
       </c>
       <c r="L49" t="n">
-        <v>177592.42</v>
+        <v>17048.98</v>
       </c>
       <c r="M49" t="n">
         <v>1.91</v>
       </c>
       <c r="N49" t="n">
-        <v>90401.0</v>
+        <v>90501.0</v>
       </c>
       <c r="O49" t="s">
-        <v>51</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B50" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C50" t="n">
-        <v>910.0</v>
+        <v>904.0</v>
       </c>
       <c r="D50" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="E50" t="s">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="F50" t="n">
         <v>1.0</v>
       </c>
       <c r="G50" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H50" t="s">
-        <v>98</v>
+        <v>51</v>
       </c>
       <c r="I50" t="n">
-        <v>27000.0</v>
+        <v>181445.0</v>
       </c>
       <c r="J50" t="n">
-        <v>990.7</v>
+        <v>3852.58</v>
       </c>
       <c r="K50" t="n">
-        <v>26009.3</v>
+        <v>177592.42</v>
       </c>
       <c r="L50" t="n">
-        <v>26009.3</v>
+        <v>177592.42</v>
       </c>
       <c r="M50" t="n">
         <v>1.91</v>
       </c>
       <c r="N50" t="n">
-        <v>91001.0</v>
+        <v>90401.0</v>
       </c>
       <c r="O50" t="s">
-        <v>98</v>
+        <v>51</v>
       </c>
     </row>
     <row r="51">
@@ -1639,54 +1645,93 @@
         <v>102</v>
       </c>
       <c r="B51" t="s">
+        <v>65</v>
+      </c>
+      <c r="C51" t="n">
+        <v>910.0</v>
+      </c>
+      <c r="D51" t="s">
+        <v>93</v>
+      </c>
+      <c r="E51" t="s">
         <v>103</v>
       </c>
-      <c r="C51" t="n">
+      <c r="F51" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G51" t="s">
+        <v>50</v>
+      </c>
+      <c r="H51" t="s">
+        <v>100</v>
+      </c>
+      <c r="I51" t="n">
+        <v>27000.0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>990.7</v>
+      </c>
+      <c r="K51" t="n">
+        <v>26009.3</v>
+      </c>
+      <c r="L51" t="n">
+        <v>26009.3</v>
+      </c>
+      <c r="M51" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="N51" t="n">
+        <v>91001.0</v>
+      </c>
+      <c r="O51" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>104</v>
+      </c>
+      <c r="B52" t="s">
+        <v>105</v>
+      </c>
+      <c r="C52" t="n">
         <v>912.0</v>
       </c>
-      <c r="D51" t="s">
-        <v>98</v>
-      </c>
-      <c r="E51" t="s">
-        <v>104</v>
-      </c>
-      <c r="F51" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G51" t="s">
-        <v>55</v>
-      </c>
-      <c r="H51" t="s">
-        <v>98</v>
-      </c>
-      <c r="I51" t="n">
+      <c r="D52" t="s">
+        <v>100</v>
+      </c>
+      <c r="E52" t="s">
+        <v>106</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G52" t="s">
+        <v>50</v>
+      </c>
+      <c r="H52" t="s">
+        <v>100</v>
+      </c>
+      <c r="I52" t="n">
         <v>1250.0</v>
       </c>
-      <c r="J51" t="n">
+      <c r="J52" t="n">
         <v>118.0</v>
       </c>
-      <c r="K51" t="n">
+      <c r="K52" t="n">
         <v>1132.0</v>
       </c>
-      <c r="L51" t="n">
+      <c r="L52" t="n">
         <v>1132.0</v>
       </c>
-      <c r="M51" t="n">
+      <c r="M52" t="n">
         <v>3.17</v>
       </c>
-      <c r="N51" t="n">
+      <c r="N52" t="n">
         <v>91201.0</v>
       </c>
-      <c r="O51" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>106</v>
+      <c r="O52" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="55">
@@ -1694,15 +1739,15 @@
         <v>107</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>108</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="57">
@@ -1715,15 +1760,15 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="s">
-        <v>17</v>
+        <v>112</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="s">
-        <v>113</v>
+        <v>17</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>114</v>
@@ -1751,6 +1796,14 @@
       </c>
       <c r="B62" s="3" t="s">
         <v>120</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dados: 2026-10-12 15:48 (108 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Jul_2026.xlsx
+++ b/xlsx/carteira_mensal/Jul_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="121">
   <si>
     <t>Acompanhamento de Carteira</t>
   </si>
@@ -75,24 +75,24 @@
     <t>Data de Criação do Projeto</t>
   </si>
   <si>
+    <t>01/07/2026 até 31/07/2026</t>
+  </si>
+  <si>
+    <t>Data de Criação do Orçamento</t>
+  </si>
+  <si>
+    <t>/  /     00:00 até   /  /     00:00</t>
+  </si>
+  <si>
+    <t>Data de Criação do Contrato</t>
+  </si>
+  <si>
     <t>/  /     até   /  /</t>
   </si>
   <si>
-    <t>Data de Criação do Orçamento</t>
-  </si>
-  <si>
-    <t>/  /     00:00 até   /  /     00:00</t>
-  </si>
-  <si>
-    <t>Data de Criação do Contrato</t>
-  </si>
-  <si>
     <t>Data de Assinatura do Contrato</t>
   </si>
   <si>
-    <t>01/07/2026 até 31/07/2026</t>
-  </si>
-  <si>
     <t>Data de Criação do Cliente</t>
   </si>
   <si>
@@ -153,42 +153,36 @@
     <t>Contrato</t>
   </si>
   <si>
-    <t>Marina Pezzotti Marques</t>
+    <t>Rafael Martins Sardinha</t>
   </si>
   <si>
     <t>Parceiro</t>
   </si>
   <si>
-    <t>17/06/26</t>
+    <t>02/07/26</t>
   </si>
   <si>
     <t>ROSANGELA PACHECO</t>
   </si>
   <si>
+    <t>Orçamento Principal</t>
+  </si>
+  <si>
+    <t>27/07/26</t>
+  </si>
+  <si>
+    <t>Daniel Teixeira</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>ERIC SERPA</t>
+  </si>
+  <si>
     <t>Orçamento 1</t>
   </si>
   <si>
-    <t>27/07/26</t>
-  </si>
-  <si>
-    <t>Rafael Martins Sardinha</t>
-  </si>
-  <si>
-    <t>02/07/26</t>
-  </si>
-  <si>
-    <t>Orçamento Principal</t>
-  </si>
-  <si>
-    <t>Daniel Teixeira</t>
-  </si>
-  <si>
-    <t>Google</t>
-  </si>
-  <si>
-    <t>ERIC SERPA</t>
-  </si>
-  <si>
     <t>06/07/26</t>
   </si>
   <si>
@@ -339,7 +333,7 @@
     <t>Quantidade de Projetos</t>
   </si>
   <si>
-    <t>22</t>
+    <t>21</t>
   </si>
   <si>
     <t>Quantidade de Orçamentos</t>
@@ -348,40 +342,40 @@
     <t>Pontuação Total</t>
   </si>
   <si>
-    <t>1.93</t>
+    <t>1.92</t>
   </si>
   <si>
     <t>Valor Total Bruto</t>
   </si>
   <si>
-    <t>1.069.425,70</t>
-  </si>
-  <si>
-    <t>752.783,44</t>
+    <t>941.558,81</t>
+  </si>
+  <si>
+    <t>657.783,44</t>
   </si>
   <si>
     <t>Valor Total Líquido</t>
   </si>
   <si>
-    <t>702.876,41</t>
+    <t>614.785,72</t>
   </si>
   <si>
     <t>Total Líquido sem o Per</t>
   </si>
   <si>
-    <t>689.117,12</t>
+    <t>611.786,80</t>
   </si>
   <si>
     <t>Total Diferença Financeira</t>
   </si>
   <si>
-    <t>49.907,03</t>
+    <t>42.997,72</t>
   </si>
   <si>
     <t>Total Adicional dos Ambientes</t>
   </si>
   <si>
-    <t>39.308,69</t>
+    <t>33.990,09</t>
   </si>
 </sst>
 </file>
@@ -450,7 +444,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:O63"/>
+  <dimension ref="A2:O62"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="53.22265625" customWidth="true" bestFit="true"/>
@@ -578,15 +572,15 @@
         <v>23</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
@@ -594,7 +588,7 @@
         <v>26</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21">
@@ -602,7 +596,7 @@
         <v>27</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22">
@@ -708,7 +702,7 @@
         <v>47</v>
       </c>
       <c r="C31" t="n">
-        <v>843.0</v>
+        <v>860.0</v>
       </c>
       <c r="D31" t="s">
         <v>48</v>
@@ -726,22 +720,22 @@
         <v>51</v>
       </c>
       <c r="I31" t="n">
-        <v>95000.0</v>
+        <v>22665.4</v>
       </c>
       <c r="J31" t="n">
-        <v>6909.31</v>
+        <v>1068.34</v>
       </c>
       <c r="K31" t="n">
-        <v>88090.69</v>
+        <v>21597.06</v>
       </c>
       <c r="L31" t="n">
-        <v>77330.32</v>
+        <v>21597.06</v>
       </c>
       <c r="M31" t="n">
-        <v>2.03</v>
+        <v>1.8</v>
       </c>
       <c r="N31" t="n">
-        <v>84301.0</v>
+        <v>86002.0</v>
       </c>
       <c r="O31" t="s">
         <v>51</v>
@@ -752,422 +746,422 @@
         <v>52</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C32" t="n">
-        <v>860.0</v>
+        <v>859.0</v>
       </c>
       <c r="D32" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E32" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="F32" t="n">
         <v>1.0</v>
       </c>
       <c r="G32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H32" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="I32" t="n">
-        <v>22665.4</v>
+        <v>38177.77</v>
       </c>
       <c r="J32" t="n">
-        <v>1068.34</v>
+        <v>987.17</v>
       </c>
       <c r="K32" t="n">
-        <v>21597.06</v>
+        <v>37190.6</v>
       </c>
       <c r="L32" t="n">
-        <v>21597.06</v>
+        <v>36349.34</v>
       </c>
       <c r="M32" t="n">
-        <v>1.8</v>
+        <v>1.96</v>
       </c>
       <c r="N32" t="n">
-        <v>86002.0</v>
+        <v>85901.0</v>
       </c>
       <c r="O32" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B33" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C33" t="n">
-        <v>859.0</v>
+        <v>862.0</v>
       </c>
       <c r="D33" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E33" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="F33" t="n">
         <v>1.0</v>
       </c>
       <c r="G33" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H33" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I33" t="n">
-        <v>38177.77</v>
+        <v>11840.44</v>
       </c>
       <c r="J33" t="n">
-        <v>987.17</v>
+        <v>434.46</v>
       </c>
       <c r="K33" t="n">
-        <v>37190.6</v>
+        <v>11405.98</v>
       </c>
       <c r="L33" t="n">
-        <v>36349.34</v>
+        <v>11405.98</v>
       </c>
       <c r="M33" t="n">
-        <v>1.96</v>
+        <v>2.23</v>
       </c>
       <c r="N33" t="n">
-        <v>85901.0</v>
+        <v>86201.0</v>
       </c>
       <c r="O33" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B34" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C34" t="n">
-        <v>862.0</v>
+        <v>861.0</v>
       </c>
       <c r="D34" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E34" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="F34" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="G34" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I34" t="n">
-        <v>11840.44</v>
+        <v>1000.0</v>
       </c>
       <c r="J34" t="n">
-        <v>434.46</v>
+        <v>48.92</v>
       </c>
       <c r="K34" t="n">
-        <v>11405.98</v>
+        <v>951.08</v>
       </c>
       <c r="L34" t="n">
-        <v>11405.98</v>
+        <v>951.08</v>
       </c>
       <c r="M34" t="n">
-        <v>2.23</v>
+        <v>3.3</v>
       </c>
       <c r="N34" t="n">
-        <v>86201.0</v>
+        <v>86102.0</v>
       </c>
       <c r="O34" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B35" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C35" t="n">
-        <v>861.0</v>
+        <v>872.0</v>
       </c>
       <c r="D35" t="s">
         <v>61</v>
       </c>
       <c r="E35" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F35" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="G35" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="H35" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="I35" t="n">
-        <v>1000.0</v>
+        <v>14700.0</v>
       </c>
       <c r="J35" t="n">
-        <v>48.92</v>
+        <v>1420.24</v>
       </c>
       <c r="K35" t="n">
-        <v>951.08</v>
+        <v>13279.76</v>
       </c>
       <c r="L35" t="n">
-        <v>951.08</v>
+        <v>13279.76</v>
       </c>
       <c r="M35" t="n">
-        <v>3.3</v>
+        <v>1.96</v>
       </c>
       <c r="N35" t="n">
-        <v>86102.0</v>
+        <v>87201.0</v>
       </c>
       <c r="O35" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" t="s">
         <v>69</v>
       </c>
-      <c r="B36" t="s">
-        <v>65</v>
-      </c>
       <c r="C36" t="n">
-        <v>872.0</v>
+        <v>873.0</v>
       </c>
       <c r="D36" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="E36" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F36" t="n">
         <v>1.0</v>
       </c>
       <c r="G36" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H36" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="I36" t="n">
-        <v>14700.0</v>
+        <v>26000.01</v>
       </c>
       <c r="J36" t="n">
-        <v>1420.24</v>
+        <v>667.09</v>
       </c>
       <c r="K36" t="n">
-        <v>13279.76</v>
+        <v>25332.92</v>
       </c>
       <c r="L36" t="n">
-        <v>13279.76</v>
+        <v>24731.18</v>
       </c>
       <c r="M36" t="n">
-        <v>1.96</v>
+        <v>1.85</v>
       </c>
       <c r="N36" t="n">
-        <v>87201.0</v>
+        <v>87301.0</v>
       </c>
       <c r="O36" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="C37" t="n">
-        <v>873.0</v>
+        <v>876.0</v>
       </c>
       <c r="D37" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E37" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F37" t="n">
         <v>1.0</v>
       </c>
       <c r="G37" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H37" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I37" t="n">
-        <v>26000.01</v>
+        <v>34000.0</v>
       </c>
       <c r="J37" t="n">
-        <v>667.09</v>
+        <v>1247.55</v>
       </c>
       <c r="K37" t="n">
-        <v>25332.92</v>
+        <v>32752.45</v>
       </c>
       <c r="L37" t="n">
-        <v>24731.18</v>
+        <v>32752.45</v>
       </c>
       <c r="M37" t="n">
-        <v>1.85</v>
+        <v>1.96</v>
       </c>
       <c r="N37" t="n">
-        <v>87301.0</v>
+        <v>87601.0</v>
       </c>
       <c r="O37" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B38" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="C38" t="n">
-        <v>876.0</v>
+        <v>882.0</v>
       </c>
       <c r="D38" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="E38" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F38" t="n">
         <v>1.0</v>
       </c>
       <c r="G38" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H38" t="s">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="I38" t="n">
-        <v>34000.0</v>
+        <v>18388.0</v>
       </c>
       <c r="J38" t="n">
-        <v>1247.55</v>
+        <v>2735.99</v>
       </c>
       <c r="K38" t="n">
-        <v>32752.45</v>
+        <v>15652.01</v>
       </c>
       <c r="L38" t="n">
-        <v>32752.45</v>
+        <v>15652.01</v>
       </c>
       <c r="M38" t="n">
-        <v>1.96</v>
+        <v>1.9</v>
       </c>
       <c r="N38" t="n">
-        <v>87601.0</v>
+        <v>88201.0</v>
       </c>
       <c r="O38" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39" t="s">
         <v>77</v>
       </c>
-      <c r="B39" t="s">
-        <v>47</v>
-      </c>
       <c r="C39" t="n">
-        <v>882.0</v>
+        <v>881.0</v>
       </c>
       <c r="D39" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E39" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="F39" t="n">
         <v>1.0</v>
       </c>
       <c r="G39" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H39" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="I39" t="n">
-        <v>18388.0</v>
+        <v>1480.0</v>
       </c>
       <c r="J39" t="n">
-        <v>2735.99</v>
+        <v>0.0</v>
       </c>
       <c r="K39" t="n">
-        <v>15652.01</v>
+        <v>1480.0</v>
       </c>
       <c r="L39" t="n">
-        <v>15652.01</v>
+        <v>1480.0</v>
       </c>
       <c r="M39" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="N39" t="n">
-        <v>88201.0</v>
+        <v>88101.0</v>
       </c>
       <c r="O39" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C40" t="n">
-        <v>881.0</v>
+        <v>880.0</v>
       </c>
       <c r="D40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E40" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="F40" t="n">
         <v>1.0</v>
       </c>
       <c r="G40" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H40" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="I40" t="n">
-        <v>1480.0</v>
+        <v>16645.87</v>
       </c>
       <c r="J40" t="n">
-        <v>0.0</v>
+        <v>4019.29</v>
       </c>
       <c r="K40" t="n">
-        <v>1480.0</v>
+        <v>12626.58</v>
       </c>
       <c r="L40" t="n">
-        <v>1480.0</v>
+        <v>12626.58</v>
       </c>
       <c r="M40" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="N40" t="n">
-        <v>88101.0</v>
+        <v>88001.0</v>
       </c>
       <c r="O40" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41">
@@ -1175,90 +1169,90 @@
         <v>81</v>
       </c>
       <c r="B41" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" t="n">
+        <v>886.0</v>
+      </c>
+      <c r="D41" t="s">
         <v>82</v>
       </c>
-      <c r="C41" t="n">
-        <v>880.0</v>
-      </c>
-      <c r="D41" t="s">
-        <v>62</v>
-      </c>
       <c r="E41" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F41" t="n">
         <v>1.0</v>
       </c>
       <c r="G41" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H41" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="I41" t="n">
-        <v>16645.87</v>
+        <v>35716.8</v>
       </c>
       <c r="J41" t="n">
-        <v>4019.29</v>
+        <v>3546.5</v>
       </c>
       <c r="K41" t="n">
-        <v>12626.58</v>
+        <v>32170.3</v>
       </c>
       <c r="L41" t="n">
-        <v>12626.58</v>
+        <v>31420.53</v>
       </c>
       <c r="M41" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="N41" t="n">
-        <v>88001.0</v>
+        <v>88601.0</v>
       </c>
       <c r="O41" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B42" t="s">
+        <v>53</v>
+      </c>
+      <c r="C42" t="n">
+        <v>884.0</v>
+      </c>
+      <c r="D42" t="s">
+        <v>82</v>
+      </c>
+      <c r="E42" t="s">
+        <v>54</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G42" t="s">
+        <v>55</v>
+      </c>
+      <c r="H42" t="s">
         <v>71</v>
       </c>
-      <c r="C42" t="n">
-        <v>886.0</v>
-      </c>
-      <c r="D42" t="s">
-        <v>84</v>
-      </c>
-      <c r="E42" t="s">
-        <v>57</v>
-      </c>
-      <c r="F42" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G42" t="s">
-        <v>50</v>
-      </c>
-      <c r="H42" t="s">
-        <v>85</v>
-      </c>
       <c r="I42" t="n">
-        <v>35716.8</v>
+        <v>102000.0</v>
       </c>
       <c r="J42" t="n">
-        <v>3546.5</v>
+        <v>12052.71</v>
       </c>
       <c r="K42" t="n">
-        <v>32170.3</v>
+        <v>89947.29</v>
       </c>
       <c r="L42" t="n">
-        <v>31420.53</v>
+        <v>89947.29</v>
       </c>
       <c r="M42" t="n">
-        <v>1.9</v>
+        <v>1.95</v>
       </c>
       <c r="N42" t="n">
-        <v>88601.0</v>
+        <v>88401.0</v>
       </c>
       <c r="O42" t="s">
         <v>85</v>
@@ -1269,140 +1263,140 @@
         <v>86</v>
       </c>
       <c r="B43" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C43" t="n">
-        <v>884.0</v>
+        <v>893.0</v>
       </c>
       <c r="D43" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E43" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F43" t="n">
         <v>1.0</v>
       </c>
       <c r="G43" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H43" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="I43" t="n">
-        <v>102000.0</v>
+        <v>1930.0</v>
       </c>
       <c r="J43" t="n">
-        <v>12052.71</v>
+        <v>55.77</v>
       </c>
       <c r="K43" t="n">
-        <v>89947.29</v>
+        <v>1874.23</v>
       </c>
       <c r="L43" t="n">
-        <v>89947.29</v>
+        <v>1874.23</v>
       </c>
       <c r="M43" t="n">
-        <v>1.95</v>
+        <v>1.91</v>
       </c>
       <c r="N43" t="n">
-        <v>88401.0</v>
+        <v>89301.0</v>
       </c>
       <c r="O43" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
+        <v>89</v>
+      </c>
+      <c r="B44" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" t="n">
+        <v>898.0</v>
+      </c>
+      <c r="D44" t="s">
         <v>88</v>
       </c>
-      <c r="B44" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44" t="n">
-        <v>893.0</v>
-      </c>
-      <c r="D44" t="s">
-        <v>89</v>
-      </c>
       <c r="E44" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F44" t="n">
         <v>1.0</v>
       </c>
       <c r="G44" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H44" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I44" t="n">
-        <v>1930.0</v>
+        <v>35000.0</v>
       </c>
       <c r="J44" t="n">
-        <v>55.77</v>
+        <v>1284.24</v>
       </c>
       <c r="K44" t="n">
-        <v>1874.23</v>
+        <v>33715.76</v>
       </c>
       <c r="L44" t="n">
-        <v>1874.23</v>
+        <v>32909.61</v>
       </c>
       <c r="M44" t="n">
-        <v>1.91</v>
+        <v>1.9</v>
       </c>
       <c r="N44" t="n">
-        <v>89301.0</v>
+        <v>89801.0</v>
       </c>
       <c r="O44" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B45" t="s">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="C45" t="n">
-        <v>898.0</v>
+        <v>901.0</v>
       </c>
       <c r="D45" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E45" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F45" t="n">
         <v>1.0</v>
       </c>
       <c r="G45" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H45" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="I45" t="n">
-        <v>35000.0</v>
+        <v>52950.0</v>
       </c>
       <c r="J45" t="n">
-        <v>1284.24</v>
+        <v>3328.95</v>
       </c>
       <c r="K45" t="n">
-        <v>33715.76</v>
+        <v>49621.05</v>
       </c>
       <c r="L45" t="n">
-        <v>32909.61</v>
+        <v>49621.05</v>
       </c>
       <c r="M45" t="n">
         <v>1.9</v>
       </c>
       <c r="N45" t="n">
-        <v>89801.0</v>
+        <v>90101.0</v>
       </c>
       <c r="O45" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
     </row>
     <row r="46">
@@ -1410,140 +1404,140 @@
         <v>95</v>
       </c>
       <c r="B46" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C46" t="n">
-        <v>901.0</v>
+        <v>900.0</v>
       </c>
       <c r="D46" t="s">
+        <v>94</v>
+      </c>
+      <c r="E46" t="s">
         <v>96</v>
       </c>
-      <c r="E46" t="s">
-        <v>66</v>
-      </c>
       <c r="F46" t="n">
         <v>1.0</v>
       </c>
       <c r="G46" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H46" t="s">
-        <v>51</v>
+        <v>94</v>
       </c>
       <c r="I46" t="n">
-        <v>52950.0</v>
+        <v>1100.0</v>
       </c>
       <c r="J46" t="n">
-        <v>3328.95</v>
+        <v>0.0</v>
       </c>
       <c r="K46" t="n">
-        <v>49621.05</v>
+        <v>1100.0</v>
       </c>
       <c r="L46" t="n">
-        <v>49621.05</v>
+        <v>1100.0</v>
       </c>
       <c r="M46" t="n">
-        <v>1.9</v>
+        <v>3.0</v>
       </c>
       <c r="N46" t="n">
-        <v>90101.0</v>
+        <v>90001.0</v>
       </c>
       <c r="O46" t="s">
-        <v>51</v>
+        <v>94</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="B47" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C47" t="n">
-        <v>900.0</v>
+        <v>907.0</v>
       </c>
       <c r="D47" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="E47" t="s">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="F47" t="n">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="G47" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H47" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="I47" t="n">
-        <v>1100.0</v>
+        <v>16223.15</v>
       </c>
       <c r="J47" t="n">
-        <v>0.0</v>
+        <v>3917.2</v>
       </c>
       <c r="K47" t="n">
-        <v>1100.0</v>
+        <v>12305.95</v>
       </c>
       <c r="L47" t="n">
-        <v>1100.0</v>
+        <v>12305.95</v>
       </c>
       <c r="M47" t="n">
-        <v>3.0</v>
+        <v>1.8</v>
       </c>
       <c r="N47" t="n">
-        <v>90001.0</v>
+        <v>90701.0</v>
       </c>
       <c r="O47" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="B48" t="s">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="C48" t="n">
-        <v>907.0</v>
+        <v>905.0</v>
       </c>
       <c r="D48" t="s">
         <v>51</v>
       </c>
       <c r="E48" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F48" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="G48" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H48" t="s">
-        <v>51</v>
+        <v>98</v>
       </c>
       <c r="I48" t="n">
-        <v>16223.15</v>
+        <v>18271.0</v>
       </c>
       <c r="J48" t="n">
-        <v>3917.2</v>
+        <v>1222.02</v>
       </c>
       <c r="K48" t="n">
-        <v>12305.95</v>
+        <v>17048.98</v>
       </c>
       <c r="L48" t="n">
-        <v>12305.95</v>
+        <v>17048.98</v>
       </c>
       <c r="M48" t="n">
-        <v>1.8</v>
+        <v>1.91</v>
       </c>
       <c r="N48" t="n">
-        <v>90701.0</v>
+        <v>90501.0</v>
       </c>
       <c r="O48" t="s">
-        <v>51</v>
+        <v>98</v>
       </c>
     </row>
     <row r="49">
@@ -1551,93 +1545,93 @@
         <v>99</v>
       </c>
       <c r="B49" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="C49" t="n">
-        <v>905.0</v>
+        <v>904.0</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
       </c>
       <c r="E49" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F49" t="n">
         <v>1.0</v>
       </c>
       <c r="G49" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H49" t="s">
-        <v>100</v>
+        <v>51</v>
       </c>
       <c r="I49" t="n">
-        <v>18271.0</v>
+        <v>181445.0</v>
       </c>
       <c r="J49" t="n">
-        <v>1222.02</v>
+        <v>3852.58</v>
       </c>
       <c r="K49" t="n">
-        <v>17048.98</v>
+        <v>177592.42</v>
       </c>
       <c r="L49" t="n">
-        <v>17048.98</v>
+        <v>177592.42</v>
       </c>
       <c r="M49" t="n">
         <v>1.91</v>
       </c>
       <c r="N49" t="n">
-        <v>90501.0</v>
+        <v>90401.0</v>
       </c>
       <c r="O49" t="s">
-        <v>100</v>
+        <v>51</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
+        <v>100</v>
+      </c>
+      <c r="B50" t="s">
+        <v>63</v>
+      </c>
+      <c r="C50" t="n">
+        <v>910.0</v>
+      </c>
+      <c r="D50" t="s">
+        <v>91</v>
+      </c>
+      <c r="E50" t="s">
         <v>101</v>
       </c>
-      <c r="B50" t="s">
-        <v>79</v>
-      </c>
-      <c r="C50" t="n">
-        <v>904.0</v>
-      </c>
-      <c r="D50" t="s">
-        <v>51</v>
-      </c>
-      <c r="E50" t="s">
-        <v>66</v>
-      </c>
       <c r="F50" t="n">
         <v>1.0</v>
       </c>
       <c r="G50" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H50" t="s">
-        <v>51</v>
+        <v>98</v>
       </c>
       <c r="I50" t="n">
-        <v>181445.0</v>
+        <v>27000.0</v>
       </c>
       <c r="J50" t="n">
-        <v>3852.58</v>
+        <v>990.7</v>
       </c>
       <c r="K50" t="n">
-        <v>177592.42</v>
+        <v>26009.3</v>
       </c>
       <c r="L50" t="n">
-        <v>177592.42</v>
+        <v>26009.3</v>
       </c>
       <c r="M50" t="n">
         <v>1.91</v>
       </c>
       <c r="N50" t="n">
-        <v>90401.0</v>
+        <v>91001.0</v>
       </c>
       <c r="O50" t="s">
-        <v>51</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51">
@@ -1645,93 +1639,54 @@
         <v>102</v>
       </c>
       <c r="B51" t="s">
-        <v>65</v>
+        <v>103</v>
       </c>
       <c r="C51" t="n">
-        <v>910.0</v>
+        <v>912.0</v>
       </c>
       <c r="D51" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E51" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F51" t="n">
         <v>1.0</v>
       </c>
       <c r="G51" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H51" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I51" t="n">
-        <v>27000.0</v>
+        <v>1250.0</v>
       </c>
       <c r="J51" t="n">
-        <v>990.7</v>
+        <v>118.0</v>
       </c>
       <c r="K51" t="n">
-        <v>26009.3</v>
+        <v>1132.0</v>
       </c>
       <c r="L51" t="n">
-        <v>26009.3</v>
+        <v>1132.0</v>
       </c>
       <c r="M51" t="n">
-        <v>1.91</v>
+        <v>3.17</v>
       </c>
       <c r="N51" t="n">
-        <v>91001.0</v>
+        <v>91201.0</v>
       </c>
       <c r="O51" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="s">
-        <v>104</v>
-      </c>
-      <c r="B52" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C52" t="n">
-        <v>912.0</v>
-      </c>
-      <c r="D52" t="s">
-        <v>100</v>
-      </c>
-      <c r="E52" t="s">
+      <c r="B54" s="3" t="s">
         <v>106</v>
-      </c>
-      <c r="F52" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G52" t="s">
-        <v>50</v>
-      </c>
-      <c r="H52" t="s">
-        <v>100</v>
-      </c>
-      <c r="I52" t="n">
-        <v>1250.0</v>
-      </c>
-      <c r="J52" t="n">
-        <v>118.0</v>
-      </c>
-      <c r="K52" t="n">
-        <v>1132.0</v>
-      </c>
-      <c r="L52" t="n">
-        <v>1132.0</v>
-      </c>
-      <c r="M52" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="N52" t="n">
-        <v>91201.0</v>
-      </c>
-      <c r="O52" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="55">
@@ -1739,15 +1694,15 @@
         <v>107</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="57">
@@ -1760,15 +1715,15 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B58" s="3" t="s">
         <v>112</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="s">
-        <v>17</v>
+        <v>113</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>114</v>
@@ -1796,14 +1751,6 @@
       </c>
       <c r="B62" s="3" t="s">
         <v>120</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>